<commit_message>
fix(xlsx): fix wrong conditional formatting
</commit_message>
<xml_diff>
--- a/Tabla_Resultados_Corrida.xlsx
+++ b/Tabla_Resultados_Corrida.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antonio\Models\mi-proyecto-anylogic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFB0AF7-A730-4F0B-A59D-03C43D4D0F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163E4BA4-AE9D-457D-9F40-2D9BD1F9366C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A923D075-8E6E-4AD4-8B2A-316AD42E9CB3}"/>
   </bookViews>
@@ -237,38 +237,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="106">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="48">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -276,16 +253,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -421,56 +388,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -516,19 +433,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -753,494 +657,7 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1326,8 +743,8 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{29BADEF3-00F3-4923-9B25-9276A2AB6AF3}" uniqueName="1" name="Dia" queryTableFieldId="1" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{7FF5DB85-B9DE-4A5F-8C22-4E66327D084E}" uniqueName="2" name="Hora" queryTableFieldId="2" dataDxfId="104"/>
+    <tableColumn id="1" xr3:uid="{29BADEF3-00F3-4923-9B25-9276A2AB6AF3}" uniqueName="1" name="Dia" queryTableFieldId="1" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{7FF5DB85-B9DE-4A5F-8C22-4E66327D084E}" uniqueName="2" name="Hora" queryTableFieldId="2" dataDxfId="46"/>
     <tableColumn id="3" xr3:uid="{06DDC69D-1405-41D2-A484-702BD6EB6B49}" uniqueName="3" name="Entradas Externo" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{EF2FE910-1170-47C3-9301-CB1EDF69007F}" uniqueName="4" name="Salidas Externo" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{CDF657CF-72AD-48AD-A9F4-18C306027810}" uniqueName="5" name="Ocupación Externo" queryTableFieldId="5"/>
@@ -1341,19 +758,19 @@
     <tableColumn id="13" xr3:uid="{CA0D0D81-2959-4048-B568-C2A3ECAE3564}" uniqueName="13" name="Salidas Total" queryTableFieldId="13"/>
     <tableColumn id="14" xr3:uid="{7662A870-E3B2-4154-B61C-1FBF71041EC3}" uniqueName="14" name="OcupTotal" queryTableFieldId="14"/>
     <tableColumn id="15" xr3:uid="{D9DFDC86-A607-4E1A-AC03-BA515BCBAFFD}" uniqueName="15" name="Rechazados acumulados" queryTableFieldId="15"/>
-    <tableColumn id="17" xr3:uid="{C1FC1DA5-EF45-4471-8849-5F495E3FF680}" uniqueName="17" name="% Utilización Total" queryTableFieldId="17" dataDxfId="103">
+    <tableColumn id="17" xr3:uid="{C1FC1DA5-EF45-4471-8849-5F495E3FF680}" uniqueName="17" name="% Utilización Total" queryTableFieldId="17" dataDxfId="45">
       <calculatedColumnFormula>+output[[#This Row],[OcupTotal]]/264</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{5E209660-3C78-463E-8A28-FB880F017BEF}" uniqueName="18" name="% Utilización Externo" queryTableFieldId="18" dataDxfId="102">
+    <tableColumn id="18" xr3:uid="{5E209660-3C78-463E-8A28-FB880F017BEF}" uniqueName="18" name="% Utilización Externo" queryTableFieldId="18" dataDxfId="44">
       <calculatedColumnFormula>+output[[#This Row],[Ocupación Externo]]/100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{A5807F5A-8F30-44BB-AB84-52E671F2A0A3}" uniqueName="19" name="% Utilización Central" queryTableFieldId="19" dataDxfId="101">
+    <tableColumn id="19" xr3:uid="{A5807F5A-8F30-44BB-AB84-52E671F2A0A3}" uniqueName="19" name="% Utilización Central" queryTableFieldId="19" dataDxfId="43">
       <calculatedColumnFormula>+output[[#This Row],[Ocupación Central]]/73</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{E58CA651-F54D-4F7B-A992-F3575454629B}" uniqueName="20" name="% Utilización Polideportivo" queryTableFieldId="20" dataDxfId="100">
+    <tableColumn id="20" xr3:uid="{E58CA651-F54D-4F7B-A992-F3575454629B}" uniqueName="20" name="% Utilización Polideportivo" queryTableFieldId="20" dataDxfId="42">
       <calculatedColumnFormula>+output[[#This Row],[Ocupación Polideportivo]]/91</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{CBA7D8CD-20EB-41E6-B1A4-A2DEF8230906}" uniqueName="21" name="Rechazados por hora" queryTableFieldId="21" dataDxfId="27">
+    <tableColumn id="21" xr3:uid="{CBA7D8CD-20EB-41E6-B1A4-A2DEF8230906}" uniqueName="21" name="Rechazados por hora" queryTableFieldId="21" dataDxfId="41">
       <calculatedColumnFormula>+output[[#This Row],[Rechazados acumulados]]-O1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1691,7 +1108,6 @@
     <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" style="2"/>
     <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -1723,13 +1139,13 @@
       <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
       <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
       <c r="L1" t="s">
@@ -1791,7 +1207,7 @@
       <c r="J2">
         <v>0</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2">
         <v>26</v>
       </c>
       <c r="L2">
@@ -1803,26 +1219,26 @@
       <c r="N2">
         <v>80</v>
       </c>
-      <c r="O2" s="2">
-        <v>0</v>
-      </c>
-      <c r="P2" s="4">
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.30303030303030304</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="Q2" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.31</v>
       </c>
-      <c r="R2" s="4">
+      <c r="R2" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.31506849315068491</v>
       </c>
-      <c r="S2" s="3">
+      <c r="S2" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.2857142857142857</v>
       </c>
-      <c r="T2" s="5">
+      <c r="T2">
         <v>0</v>
       </c>
     </row>
@@ -1857,7 +1273,7 @@
       <c r="J3">
         <v>0</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3">
         <v>46</v>
       </c>
       <c r="L3">
@@ -1872,23 +1288,23 @@
       <c r="O3">
         <v>1</v>
       </c>
-      <c r="P3" s="4">
+      <c r="P3" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.54545454545454541</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="Q3" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.57534246575342463</v>
       </c>
-      <c r="S3" s="3">
+      <c r="S3" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.50549450549450547</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3">
         <f>+output[[#This Row],[Rechazados acumulados]]-O2</f>
         <v>1</v>
       </c>
@@ -1924,7 +1340,7 @@
       <c r="J4">
         <v>0</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4">
         <v>60</v>
       </c>
       <c r="L4">
@@ -1939,23 +1355,23 @@
       <c r="O4">
         <v>1</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.73106060606060608</v>
       </c>
-      <c r="Q4" s="3">
+      <c r="Q4" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.75</v>
       </c>
-      <c r="R4" s="3">
+      <c r="R4" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.79452054794520544</v>
       </c>
-      <c r="S4" s="3">
+      <c r="S4" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.65934065934065933</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4">
         <f>+output[[#This Row],[Rechazados acumulados]]-O3</f>
         <v>0</v>
       </c>
@@ -1991,7 +1407,7 @@
       <c r="J5">
         <v>5</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5">
         <v>67</v>
       </c>
       <c r="L5">
@@ -2006,23 +1422,23 @@
       <c r="O5">
         <v>1</v>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.85227272727272729</v>
       </c>
-      <c r="Q5" s="3">
+      <c r="Q5" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.94</v>
       </c>
-      <c r="R5" s="3">
+      <c r="R5" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.87671232876712324</v>
       </c>
-      <c r="S5" s="3">
+      <c r="S5" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.73626373626373631</v>
       </c>
-      <c r="T5" s="5">
+      <c r="T5">
         <f>+output[[#This Row],[Rechazados acumulados]]-O4</f>
         <v>0</v>
       </c>
@@ -2058,7 +1474,7 @@
       <c r="J6">
         <v>11</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6">
         <v>71</v>
       </c>
       <c r="L6">
@@ -2073,23 +1489,23 @@
       <c r="O6">
         <v>1</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.85984848484848486</v>
       </c>
-      <c r="Q6" s="3">
+      <c r="Q6" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.95</v>
       </c>
-      <c r="R6" s="3">
+      <c r="R6" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.83561643835616439</v>
       </c>
-      <c r="S6" s="3">
+      <c r="S6" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.78021978021978022</v>
       </c>
-      <c r="T6" s="5">
+      <c r="T6">
         <f>+output[[#This Row],[Rechazados acumulados]]-O5</f>
         <v>0</v>
       </c>
@@ -2125,7 +1541,7 @@
       <c r="J7">
         <v>16</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7">
         <v>64</v>
       </c>
       <c r="L7">
@@ -2140,23 +1556,23 @@
       <c r="O7">
         <v>1</v>
       </c>
-      <c r="P7" s="4">
+      <c r="P7" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.76515151515151514</v>
       </c>
-      <c r="Q7" s="3">
+      <c r="Q7" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.85</v>
       </c>
-      <c r="R7" s="3">
+      <c r="R7" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.72602739726027399</v>
       </c>
-      <c r="S7" s="3">
+      <c r="S7" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.70329670329670335</v>
       </c>
-      <c r="T7" s="5">
+      <c r="T7">
         <f>+output[[#This Row],[Rechazados acumulados]]-O6</f>
         <v>0</v>
       </c>
@@ -2192,7 +1608,7 @@
       <c r="J8">
         <v>17</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8">
         <v>59</v>
       </c>
       <c r="L8">
@@ -2207,23 +1623,23 @@
       <c r="O8">
         <v>1</v>
       </c>
-      <c r="P8" s="4">
+      <c r="P8" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.68560606060606055</v>
       </c>
-      <c r="Q8" s="3">
+      <c r="Q8" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.73</v>
       </c>
-      <c r="R8" s="3">
+      <c r="R8" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.67123287671232879</v>
       </c>
-      <c r="S8" s="3">
+      <c r="S8" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.64835164835164838</v>
       </c>
-      <c r="T8" s="5">
+      <c r="T8">
         <f>+output[[#This Row],[Rechazados acumulados]]-O7</f>
         <v>0</v>
       </c>
@@ -2259,7 +1675,7 @@
       <c r="J9">
         <v>12</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9">
         <v>61</v>
       </c>
       <c r="L9">
@@ -2274,23 +1690,23 @@
       <c r="O9">
         <v>1</v>
       </c>
-      <c r="P9" s="4">
+      <c r="P9" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.64015151515151514</v>
       </c>
-      <c r="Q9" s="3">
+      <c r="Q9" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.59</v>
       </c>
-      <c r="R9" s="4">
+      <c r="R9" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.67123287671232879</v>
       </c>
-      <c r="S9" s="3">
+      <c r="S9" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.67032967032967028</v>
       </c>
-      <c r="T9" s="5">
+      <c r="T9">
         <f>+output[[#This Row],[Rechazados acumulados]]-O8</f>
         <v>0</v>
       </c>
@@ -2326,7 +1742,7 @@
       <c r="J10">
         <v>16</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10">
         <v>58</v>
       </c>
       <c r="L10">
@@ -2341,23 +1757,23 @@
       <c r="O10">
         <v>1</v>
       </c>
-      <c r="P10" s="4">
+      <c r="P10" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.61742424242424243</v>
       </c>
-      <c r="Q10" s="3">
+      <c r="Q10" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="R10" s="3">
+      <c r="R10" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.67123287671232879</v>
       </c>
-      <c r="S10" s="3">
+      <c r="S10" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.63736263736263732</v>
       </c>
-      <c r="T10" s="5">
+      <c r="T10">
         <f>+output[[#This Row],[Rechazados acumulados]]-O9</f>
         <v>0</v>
       </c>
@@ -2393,7 +1809,7 @@
       <c r="J11">
         <v>13</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11">
         <v>57</v>
       </c>
       <c r="L11">
@@ -2408,23 +1824,23 @@
       <c r="O11">
         <v>1</v>
       </c>
-      <c r="P11" s="4">
+      <c r="P11" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.60606060606060608</v>
       </c>
-      <c r="Q11" s="3">
+      <c r="Q11" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="R11" s="3">
+      <c r="R11" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.64383561643835618</v>
       </c>
-      <c r="S11" s="3">
+      <c r="S11" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.62637362637362637</v>
       </c>
-      <c r="T11" s="5">
+      <c r="T11">
         <f>+output[[#This Row],[Rechazados acumulados]]-O10</f>
         <v>0</v>
       </c>
@@ -2460,7 +1876,7 @@
       <c r="J12">
         <v>10</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12">
         <v>77</v>
       </c>
       <c r="L12">
@@ -2475,23 +1891,23 @@
       <c r="O12">
         <v>2</v>
       </c>
-      <c r="P12" s="4">
+      <c r="P12" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.81060606060606055</v>
       </c>
-      <c r="Q12" s="3">
+      <c r="Q12" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.78</v>
       </c>
-      <c r="R12" s="3">
+      <c r="R12" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.80821917808219179</v>
       </c>
-      <c r="S12" s="3">
+      <c r="S12" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.84615384615384615</v>
       </c>
-      <c r="T12" s="5">
+      <c r="T12">
         <f>+output[[#This Row],[Rechazados acumulados]]-O11</f>
         <v>1</v>
       </c>
@@ -2527,7 +1943,7 @@
       <c r="J13">
         <v>13</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13">
         <v>91</v>
       </c>
       <c r="L13">
@@ -2542,23 +1958,23 @@
       <c r="O13">
         <v>4</v>
       </c>
-      <c r="P13" s="4">
+      <c r="P13" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.98106060606060608</v>
       </c>
-      <c r="Q13" s="3">
+      <c r="Q13" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.98</v>
       </c>
-      <c r="R13" s="3">
+      <c r="R13" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.95890410958904104</v>
       </c>
-      <c r="S13" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T13" s="5">
+      <c r="S13" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T13">
         <f>+output[[#This Row],[Rechazados acumulados]]-O12</f>
         <v>2</v>
       </c>
@@ -2594,7 +2010,7 @@
       <c r="J14">
         <v>14</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14">
         <v>91</v>
       </c>
       <c r="L14">
@@ -2609,23 +2025,23 @@
       <c r="O14">
         <v>4</v>
       </c>
-      <c r="P14" s="4">
-        <f>+output[[#This Row],[OcupTotal]]/264</f>
-        <v>1</v>
-      </c>
-      <c r="Q14" s="3">
-        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
-        <v>1</v>
-      </c>
-      <c r="R14" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S14" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T14" s="5">
+      <c r="P14" s="2">
+        <f>+output[[#This Row],[OcupTotal]]/264</f>
+        <v>1</v>
+      </c>
+      <c r="Q14" s="2">
+        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
+        <v>1</v>
+      </c>
+      <c r="R14" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S14" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T14">
         <f>+output[[#This Row],[Rechazados acumulados]]-O13</f>
         <v>0</v>
       </c>
@@ -2661,7 +2077,7 @@
       <c r="J15">
         <v>12</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15">
         <v>91</v>
       </c>
       <c r="L15">
@@ -2676,23 +2092,23 @@
       <c r="O15">
         <v>4</v>
       </c>
-      <c r="P15" s="4">
+      <c r="P15" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.96969696969696972</v>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.92</v>
       </c>
-      <c r="R15" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S15" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T15" s="5">
+      <c r="R15" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S15" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T15">
         <f>+output[[#This Row],[Rechazados acumulados]]-O14</f>
         <v>0</v>
       </c>
@@ -2728,7 +2144,7 @@
       <c r="J16">
         <v>20</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16">
         <v>81</v>
       </c>
       <c r="L16">
@@ -2743,23 +2159,23 @@
       <c r="O16">
         <v>4</v>
       </c>
-      <c r="P16" s="4">
+      <c r="P16" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.87121212121212122</v>
       </c>
-      <c r="Q16" s="3">
+      <c r="Q16" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.82</v>
       </c>
-      <c r="R16" s="3">
+      <c r="R16" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.9178082191780822</v>
       </c>
-      <c r="S16" s="3">
+      <c r="S16" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.89010989010989006</v>
       </c>
-      <c r="T16" s="5">
+      <c r="T16">
         <f>+output[[#This Row],[Rechazados acumulados]]-O15</f>
         <v>0</v>
       </c>
@@ -2822,11 +2238,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.65753424657534243</v>
       </c>
-      <c r="S17" s="5">
+      <c r="S17">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.64835164835164838</v>
       </c>
-      <c r="T17" s="5">
+      <c r="T17">
         <f>+output[[#This Row],[Rechazados acumulados]]-O16</f>
         <v>0</v>
       </c>
@@ -2889,11 +2305,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.42465753424657532</v>
       </c>
-      <c r="S18" s="5">
+      <c r="S18">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.37362637362637363</v>
       </c>
-      <c r="T18" s="5">
+      <c r="T18">
         <f>+output[[#This Row],[Rechazados acumulados]]-O17</f>
         <v>0</v>
       </c>
@@ -2956,11 +2372,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.19178082191780821</v>
       </c>
-      <c r="S19" s="5">
+      <c r="S19">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.26373626373626374</v>
       </c>
-      <c r="T19" s="5">
+      <c r="T19">
         <f>+output[[#This Row],[Rechazados acumulados]]-O18</f>
         <v>0</v>
       </c>
@@ -3023,11 +2439,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>9.5890410958904104E-2</v>
       </c>
-      <c r="S20" s="5">
+      <c r="S20">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.15384615384615385</v>
       </c>
-      <c r="T20" s="5">
+      <c r="T20">
         <f>+output[[#This Row],[Rechazados acumulados]]-O19</f>
         <v>0</v>
       </c>
@@ -3090,11 +2506,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>1.3698630136986301E-2</v>
       </c>
-      <c r="S21" s="5">
+      <c r="S21">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>6.5934065934065936E-2</v>
       </c>
-      <c r="T21" s="5">
+      <c r="T21">
         <f>+output[[#This Row],[Rechazados acumulados]]-O20</f>
         <v>0</v>
       </c>
@@ -3157,11 +2573,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0</v>
       </c>
-      <c r="S22" s="5">
+      <c r="S22">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>1.098901098901099E-2</v>
       </c>
-      <c r="T22" s="5">
+      <c r="T22">
         <f>+output[[#This Row],[Rechazados acumulados]]-O21</f>
         <v>0</v>
       </c>
@@ -3197,7 +2613,7 @@
       <c r="J23">
         <v>0</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23">
         <v>38</v>
       </c>
       <c r="L23">
@@ -3212,23 +2628,23 @@
       <c r="O23">
         <v>10</v>
       </c>
-      <c r="P23" s="4">
+      <c r="P23" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.32196969696969696</v>
       </c>
-      <c r="Q23" s="3">
+      <c r="Q23" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.28999999999999998</v>
       </c>
-      <c r="R23" s="3">
+      <c r="R23" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.24657534246575341</v>
       </c>
-      <c r="S23" s="3">
+      <c r="S23" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.4175824175824176</v>
       </c>
-      <c r="T23" s="5">
+      <c r="T23">
         <f>+output[[#This Row],[Rechazados acumulados]]-O22</f>
         <v>6</v>
       </c>
@@ -3264,7 +2680,7 @@
       <c r="J24">
         <v>0</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24">
         <v>55</v>
       </c>
       <c r="L24">
@@ -3279,23 +2695,23 @@
       <c r="O24">
         <v>10</v>
       </c>
-      <c r="P24" s="4">
+      <c r="P24" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.57954545454545459</v>
       </c>
-      <c r="Q24" s="3">
+      <c r="Q24" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.61</v>
       </c>
-      <c r="R24" s="3">
+      <c r="R24" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.50684931506849318</v>
       </c>
-      <c r="S24" s="3">
+      <c r="S24" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.60439560439560436</v>
       </c>
-      <c r="T24" s="5">
+      <c r="T24">
         <f>+output[[#This Row],[Rechazados acumulados]]-O23</f>
         <v>0</v>
       </c>
@@ -3331,7 +2747,7 @@
       <c r="J25">
         <v>0</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25">
         <v>64</v>
       </c>
       <c r="L25">
@@ -3346,23 +2762,23 @@
       <c r="O25">
         <v>10</v>
       </c>
-      <c r="P25" s="4">
+      <c r="P25" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.71969696969696972</v>
       </c>
-      <c r="Q25" s="3">
+      <c r="Q25" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.78</v>
       </c>
-      <c r="R25" s="3">
+      <c r="R25" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.65753424657534243</v>
       </c>
-      <c r="S25" s="3">
+      <c r="S25" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.70329670329670335</v>
       </c>
-      <c r="T25" s="5">
+      <c r="T25">
         <f>+output[[#This Row],[Rechazados acumulados]]-O24</f>
         <v>0</v>
       </c>
@@ -3398,7 +2814,7 @@
       <c r="J26">
         <v>6</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26">
         <v>69</v>
       </c>
       <c r="L26">
@@ -3413,23 +2829,23 @@
       <c r="O26">
         <v>10</v>
       </c>
-      <c r="P26" s="4">
+      <c r="P26" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.78787878787878785</v>
       </c>
-      <c r="Q26" s="3">
+      <c r="Q26" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.86</v>
       </c>
-      <c r="R26" s="3">
+      <c r="R26" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.72602739726027399</v>
       </c>
-      <c r="S26" s="3">
+      <c r="S26" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.75824175824175821</v>
       </c>
-      <c r="T26" s="5">
+      <c r="T26">
         <f>+output[[#This Row],[Rechazados acumulados]]-O25</f>
         <v>0</v>
       </c>
@@ -3465,7 +2881,7 @@
       <c r="J27">
         <v>14</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27">
         <v>64</v>
       </c>
       <c r="L27">
@@ -3480,23 +2896,23 @@
       <c r="O27">
         <v>10</v>
       </c>
-      <c r="P27" s="4">
+      <c r="P27" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.78030303030303028</v>
       </c>
-      <c r="Q27" s="3">
+      <c r="Q27" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.86</v>
       </c>
-      <c r="R27" s="3">
+      <c r="R27" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.76712328767123283</v>
       </c>
-      <c r="S27" s="3">
+      <c r="S27" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.70329670329670335</v>
       </c>
-      <c r="T27" s="5">
+      <c r="T27">
         <f>+output[[#This Row],[Rechazados acumulados]]-O26</f>
         <v>0</v>
       </c>
@@ -3532,7 +2948,7 @@
       <c r="J28">
         <v>17</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28">
         <v>57</v>
       </c>
       <c r="L28">
@@ -3547,23 +2963,23 @@
       <c r="O28">
         <v>10</v>
       </c>
-      <c r="P28" s="4">
+      <c r="P28" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.70454545454545459</v>
       </c>
-      <c r="Q28" s="3">
+      <c r="Q28" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.78</v>
       </c>
-      <c r="R28" s="3">
+      <c r="R28" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.69863013698630139</v>
       </c>
-      <c r="S28" s="3">
+      <c r="S28" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.62637362637362637</v>
       </c>
-      <c r="T28" s="5">
+      <c r="T28">
         <f>+output[[#This Row],[Rechazados acumulados]]-O27</f>
         <v>0</v>
       </c>
@@ -3599,7 +3015,7 @@
       <c r="J29">
         <v>15</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29">
         <v>50</v>
       </c>
       <c r="L29">
@@ -3614,23 +3030,23 @@
       <c r="O29">
         <v>10</v>
       </c>
-      <c r="P29" s="4">
+      <c r="P29" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.625</v>
       </c>
-      <c r="Q29" s="3">
+      <c r="Q29" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.74</v>
       </c>
-      <c r="R29" s="3">
+      <c r="R29" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.56164383561643838</v>
       </c>
-      <c r="S29" s="3">
+      <c r="S29" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.5494505494505495</v>
       </c>
-      <c r="T29" s="5">
+      <c r="T29">
         <f>+output[[#This Row],[Rechazados acumulados]]-O28</f>
         <v>0</v>
       </c>
@@ -3666,7 +3082,7 @@
       <c r="J30">
         <v>16</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30">
         <v>55</v>
       </c>
       <c r="L30">
@@ -3681,23 +3097,23 @@
       <c r="O30">
         <v>10</v>
       </c>
-      <c r="P30" s="4">
+      <c r="P30" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.61363636363636365</v>
       </c>
-      <c r="Q30" s="3">
+      <c r="Q30" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.64</v>
       </c>
-      <c r="R30" s="3">
+      <c r="R30" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.58904109589041098</v>
       </c>
-      <c r="S30" s="3">
+      <c r="S30" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.60439560439560436</v>
       </c>
-      <c r="T30" s="5">
+      <c r="T30">
         <f>+output[[#This Row],[Rechazados acumulados]]-O29</f>
         <v>0</v>
       </c>
@@ -3733,7 +3149,7 @@
       <c r="J31">
         <v>11</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31">
         <v>57</v>
       </c>
       <c r="L31">
@@ -3748,23 +3164,23 @@
       <c r="O31">
         <v>10</v>
       </c>
-      <c r="P31" s="4">
+      <c r="P31" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.58333333333333337</v>
       </c>
-      <c r="Q31" s="3">
+      <c r="Q31" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.61</v>
       </c>
-      <c r="R31" s="3">
+      <c r="R31" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.49315068493150682</v>
       </c>
-      <c r="S31" s="3">
+      <c r="S31" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.62637362637362637</v>
       </c>
-      <c r="T31" s="5">
+      <c r="T31">
         <f>+output[[#This Row],[Rechazados acumulados]]-O30</f>
         <v>0</v>
       </c>
@@ -3800,7 +3216,7 @@
       <c r="J32">
         <v>8</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32">
         <v>65</v>
       </c>
       <c r="L32">
@@ -3815,23 +3231,23 @@
       <c r="O32">
         <v>10</v>
       </c>
-      <c r="P32" s="4">
+      <c r="P32" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.61363636363636365</v>
       </c>
-      <c r="Q32" s="3">
+      <c r="Q32" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="R32" s="3">
+      <c r="R32" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.56164383561643838</v>
       </c>
-      <c r="S32" s="3">
+      <c r="S32" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.7142857142857143</v>
       </c>
-      <c r="T32" s="5">
+      <c r="T32">
         <f>+output[[#This Row],[Rechazados acumulados]]-O31</f>
         <v>0</v>
       </c>
@@ -3867,7 +3283,7 @@
       <c r="J33">
         <v>13</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33">
         <v>88</v>
       </c>
       <c r="L33">
@@ -3882,23 +3298,23 @@
       <c r="O33">
         <v>13</v>
       </c>
-      <c r="P33" s="4">
+      <c r="P33" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.84469696969696972</v>
       </c>
-      <c r="Q33" s="3">
+      <c r="Q33" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.73</v>
       </c>
-      <c r="R33" s="3">
+      <c r="R33" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.84931506849315064</v>
       </c>
-      <c r="S33" s="3">
+      <c r="S33" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.96703296703296704</v>
       </c>
-      <c r="T33" s="5">
+      <c r="T33">
         <f>+output[[#This Row],[Rechazados acumulados]]-O32</f>
         <v>3</v>
       </c>
@@ -3934,7 +3350,7 @@
       <c r="J34">
         <v>12</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34">
         <v>91</v>
       </c>
       <c r="L34">
@@ -3949,23 +3365,23 @@
       <c r="O34">
         <v>16</v>
       </c>
-      <c r="P34" s="4">
+      <c r="P34" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.99242424242424243</v>
       </c>
-      <c r="Q34" s="3">
+      <c r="Q34" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.98</v>
       </c>
-      <c r="R34" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S34" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T34" s="5">
+      <c r="R34" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S34" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T34">
         <f>+output[[#This Row],[Rechazados acumulados]]-O33</f>
         <v>3</v>
       </c>
@@ -4001,7 +3417,7 @@
       <c r="J35">
         <v>8</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35">
         <v>91</v>
       </c>
       <c r="L35">
@@ -4016,23 +3432,23 @@
       <c r="O35">
         <v>16</v>
       </c>
-      <c r="P35" s="4">
-        <f>+output[[#This Row],[OcupTotal]]/264</f>
-        <v>1</v>
-      </c>
-      <c r="Q35" s="3">
-        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
-        <v>1</v>
-      </c>
-      <c r="R35" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S35" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T35" s="5">
+      <c r="P35" s="2">
+        <f>+output[[#This Row],[OcupTotal]]/264</f>
+        <v>1</v>
+      </c>
+      <c r="Q35" s="2">
+        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
+        <v>1</v>
+      </c>
+      <c r="R35" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S35" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T35">
         <f>+output[[#This Row],[Rechazados acumulados]]-O34</f>
         <v>0</v>
       </c>
@@ -4068,7 +3484,7 @@
       <c r="J36">
         <v>18</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36">
         <v>91</v>
       </c>
       <c r="L36">
@@ -4083,23 +3499,23 @@
       <c r="O36">
         <v>16</v>
       </c>
-      <c r="P36" s="4">
-        <f>+output[[#This Row],[OcupTotal]]/264</f>
-        <v>1</v>
-      </c>
-      <c r="Q36" s="3">
-        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
-        <v>1</v>
-      </c>
-      <c r="R36" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S36" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T36" s="5">
+      <c r="P36" s="2">
+        <f>+output[[#This Row],[OcupTotal]]/264</f>
+        <v>1</v>
+      </c>
+      <c r="Q36" s="2">
+        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
+        <v>1</v>
+      </c>
+      <c r="R36" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S36" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T36">
         <f>+output[[#This Row],[Rechazados acumulados]]-O35</f>
         <v>0</v>
       </c>
@@ -4135,7 +3551,7 @@
       <c r="J37">
         <v>32</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37">
         <v>81</v>
       </c>
       <c r="L37">
@@ -4150,23 +3566,23 @@
       <c r="O37">
         <v>16</v>
       </c>
-      <c r="P37" s="4">
+      <c r="P37" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.94318181818181823</v>
       </c>
-      <c r="Q37" s="3">
+      <c r="Q37" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.95</v>
       </c>
-      <c r="R37" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S37" s="3">
+      <c r="R37" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S37" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.89010989010989006</v>
       </c>
-      <c r="T37" s="5">
+      <c r="T37">
         <f>+output[[#This Row],[Rechazados acumulados]]-O36</f>
         <v>0</v>
       </c>
@@ -4229,11 +3645,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.75342465753424659</v>
       </c>
-      <c r="S38" s="5">
+      <c r="S38">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.72527472527472525</v>
       </c>
-      <c r="T38" s="5">
+      <c r="T38">
         <f>+output[[#This Row],[Rechazados acumulados]]-O37</f>
         <v>0</v>
       </c>
@@ -4296,11 +3712,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.46575342465753422</v>
       </c>
-      <c r="S39" s="5">
+      <c r="S39">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.50549450549450547</v>
       </c>
-      <c r="T39" s="5">
+      <c r="T39">
         <f>+output[[#This Row],[Rechazados acumulados]]-O38</f>
         <v>0</v>
       </c>
@@ -4363,11 +3779,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.36986301369863012</v>
       </c>
-      <c r="S40" s="5">
+      <c r="S40">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.30769230769230771</v>
       </c>
-      <c r="T40" s="5">
+      <c r="T40">
         <f>+output[[#This Row],[Rechazados acumulados]]-O39</f>
         <v>0</v>
       </c>
@@ -4430,11 +3846,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.15068493150684931</v>
       </c>
-      <c r="S41" s="5">
+      <c r="S41">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.15384615384615385</v>
       </c>
-      <c r="T41" s="5">
+      <c r="T41">
         <f>+output[[#This Row],[Rechazados acumulados]]-O40</f>
         <v>0</v>
       </c>
@@ -4497,11 +3913,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>5.4794520547945202E-2</v>
       </c>
-      <c r="S42" s="5">
+      <c r="S42">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>7.6923076923076927E-2</v>
       </c>
-      <c r="T42" s="5">
+      <c r="T42">
         <f>+output[[#This Row],[Rechazados acumulados]]-O41</f>
         <v>0</v>
       </c>
@@ -4564,11 +3980,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>1.3698630136986301E-2</v>
       </c>
-      <c r="S43" s="5">
+      <c r="S43">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>1.098901098901099E-2</v>
       </c>
-      <c r="T43" s="5">
+      <c r="T43">
         <f>+output[[#This Row],[Rechazados acumulados]]-O42</f>
         <v>0</v>
       </c>
@@ -4631,11 +4047,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>1.3698630136986301E-2</v>
       </c>
-      <c r="S44" s="5">
+      <c r="S44">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>1.098901098901099E-2</v>
       </c>
-      <c r="T44" s="5">
+      <c r="T44">
         <f>+output[[#This Row],[Rechazados acumulados]]-O43</f>
         <v>0</v>
       </c>
@@ -4698,11 +4114,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>1.3698630136986301E-2</v>
       </c>
-      <c r="S45" s="5">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>0</v>
-      </c>
-      <c r="T45" s="5">
+      <c r="S45">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>0</v>
+      </c>
+      <c r="T45">
         <f>+output[[#This Row],[Rechazados acumulados]]-O44</f>
         <v>0</v>
       </c>
@@ -4738,7 +4154,7 @@
       <c r="J46">
         <v>0</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46">
         <v>21</v>
       </c>
       <c r="L46">
@@ -4753,23 +4169,23 @@
       <c r="O46">
         <v>17</v>
       </c>
-      <c r="P46" s="4">
+      <c r="P46" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.29166666666666669</v>
       </c>
-      <c r="Q46" s="3">
+      <c r="Q46" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.28000000000000003</v>
       </c>
-      <c r="R46" s="3">
+      <c r="R46" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.38356164383561642</v>
       </c>
-      <c r="S46" s="3">
+      <c r="S46" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.23076923076923078</v>
       </c>
-      <c r="T46" s="5">
+      <c r="T46">
         <f>+output[[#This Row],[Rechazados acumulados]]-O45</f>
         <v>1</v>
       </c>
@@ -4805,7 +4221,7 @@
       <c r="J47">
         <v>0</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47">
         <v>46</v>
       </c>
       <c r="L47">
@@ -4820,23 +4236,23 @@
       <c r="O47">
         <v>17</v>
       </c>
-      <c r="P47" s="4">
+      <c r="P47" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.61363636363636365</v>
       </c>
-      <c r="Q47" s="3">
+      <c r="Q47" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.65</v>
       </c>
-      <c r="R47" s="3">
+      <c r="R47" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.69863013698630139</v>
       </c>
-      <c r="S47" s="3">
+      <c r="S47" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.50549450549450547</v>
       </c>
-      <c r="T47" s="5">
+      <c r="T47">
         <f>+output[[#This Row],[Rechazados acumulados]]-O46</f>
         <v>0</v>
       </c>
@@ -4872,7 +4288,7 @@
       <c r="J48">
         <v>0</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48">
         <v>63</v>
       </c>
       <c r="L48">
@@ -4887,23 +4303,23 @@
       <c r="O48">
         <v>17</v>
       </c>
-      <c r="P48" s="4">
+      <c r="P48" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.75</v>
       </c>
-      <c r="Q48" s="3">
+      <c r="Q48" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.78</v>
       </c>
-      <c r="R48" s="3">
+      <c r="R48" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.78082191780821919</v>
       </c>
-      <c r="S48" s="3">
+      <c r="S48" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.69230769230769229</v>
       </c>
-      <c r="T48" s="5">
+      <c r="T48">
         <f>+output[[#This Row],[Rechazados acumulados]]-O47</f>
         <v>0</v>
       </c>
@@ -4939,7 +4355,7 @@
       <c r="J49">
         <v>5</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49">
         <v>73</v>
       </c>
       <c r="L49">
@@ -4954,23 +4370,23 @@
       <c r="O49">
         <v>17</v>
       </c>
-      <c r="P49" s="4">
+      <c r="P49" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.84090909090909094</v>
       </c>
-      <c r="Q49" s="3">
+      <c r="Q49" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.89</v>
       </c>
-      <c r="R49" s="3">
+      <c r="R49" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.82191780821917804</v>
       </c>
-      <c r="S49" s="3">
+      <c r="S49" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.80219780219780223</v>
       </c>
-      <c r="T49" s="5">
+      <c r="T49">
         <f>+output[[#This Row],[Rechazados acumulados]]-O48</f>
         <v>0</v>
       </c>
@@ -5006,7 +4422,7 @@
       <c r="J50">
         <v>9</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50">
         <v>77</v>
       </c>
       <c r="L50">
@@ -5021,23 +4437,23 @@
       <c r="O50">
         <v>17</v>
       </c>
-      <c r="P50" s="4">
+      <c r="P50" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.85227272727272729</v>
       </c>
-      <c r="Q50" s="3">
+      <c r="Q50" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.94</v>
       </c>
-      <c r="R50" s="3">
+      <c r="R50" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.73972602739726023</v>
       </c>
-      <c r="S50" s="3">
+      <c r="S50" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.84615384615384615</v>
       </c>
-      <c r="T50" s="5">
+      <c r="T50">
         <f>+output[[#This Row],[Rechazados acumulados]]-O49</f>
         <v>0</v>
       </c>
@@ -5073,7 +4489,7 @@
       <c r="J51">
         <v>11</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51">
         <v>73</v>
       </c>
       <c r="L51">
@@ -5088,23 +4504,23 @@
       <c r="O51">
         <v>17</v>
       </c>
-      <c r="P51" s="4">
+      <c r="P51" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.78030303030303028</v>
       </c>
-      <c r="Q51" s="3">
+      <c r="Q51" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.82</v>
       </c>
-      <c r="R51" s="3">
+      <c r="R51" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.69863013698630139</v>
       </c>
-      <c r="S51" s="3">
+      <c r="S51" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.80219780219780223</v>
       </c>
-      <c r="T51" s="5">
+      <c r="T51">
         <f>+output[[#This Row],[Rechazados acumulados]]-O50</f>
         <v>0</v>
       </c>
@@ -5140,7 +4556,7 @@
       <c r="J52">
         <v>29</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52">
         <v>50</v>
       </c>
       <c r="L52">
@@ -5155,23 +4571,23 @@
       <c r="O52">
         <v>17</v>
       </c>
-      <c r="P52" s="4">
+      <c r="P52" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.63257575757575757</v>
       </c>
-      <c r="Q52" s="3">
+      <c r="Q52" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.74</v>
       </c>
-      <c r="R52" s="3">
+      <c r="R52" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.58904109589041098</v>
       </c>
-      <c r="S52" s="3">
+      <c r="S52" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.5494505494505495</v>
       </c>
-      <c r="T52" s="5">
+      <c r="T52">
         <f>+output[[#This Row],[Rechazados acumulados]]-O51</f>
         <v>0</v>
       </c>
@@ -5207,7 +4623,7 @@
       <c r="J53">
         <v>17</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53">
         <v>44</v>
       </c>
       <c r="L53">
@@ -5222,23 +4638,23 @@
       <c r="O53">
         <v>17</v>
       </c>
-      <c r="P53" s="4">
+      <c r="P53" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.55681818181818177</v>
       </c>
-      <c r="Q53" s="3">
+      <c r="Q53" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.63</v>
       </c>
-      <c r="R53" s="3">
+      <c r="R53" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.54794520547945202</v>
       </c>
-      <c r="S53" s="3">
+      <c r="S53" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.48351648351648352</v>
       </c>
-      <c r="T53" s="5">
+      <c r="T53">
         <f>+output[[#This Row],[Rechazados acumulados]]-O52</f>
         <v>0</v>
       </c>
@@ -5274,7 +4690,7 @@
       <c r="J54">
         <v>11</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54">
         <v>50</v>
       </c>
       <c r="L54">
@@ -5289,23 +4705,23 @@
       <c r="O54">
         <v>17</v>
       </c>
-      <c r="P54" s="4">
+      <c r="P54" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.53787878787878785</v>
       </c>
-      <c r="Q54" s="3">
+      <c r="Q54" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.52</v>
       </c>
-      <c r="R54" s="3">
+      <c r="R54" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.54794520547945202</v>
       </c>
-      <c r="S54" s="3">
+      <c r="S54" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.5494505494505495</v>
       </c>
-      <c r="T54" s="5">
+      <c r="T54">
         <f>+output[[#This Row],[Rechazados acumulados]]-O53</f>
         <v>0</v>
       </c>
@@ -5341,7 +4757,7 @@
       <c r="J55">
         <v>11</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55">
         <v>46</v>
       </c>
       <c r="L55">
@@ -5356,23 +4772,23 @@
       <c r="O55">
         <v>17</v>
       </c>
-      <c r="P55" s="4">
+      <c r="P55" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.54166666666666663</v>
       </c>
-      <c r="Q55" s="3">
+      <c r="Q55" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="R55" s="3">
+      <c r="R55" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.56164383561643838</v>
       </c>
-      <c r="S55" s="3">
+      <c r="S55" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.50549450549450547</v>
       </c>
-      <c r="T55" s="5">
+      <c r="T55">
         <f>+output[[#This Row],[Rechazados acumulados]]-O54</f>
         <v>0</v>
       </c>
@@ -5408,7 +4824,7 @@
       <c r="J56">
         <v>6</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56">
         <v>69</v>
       </c>
       <c r="L56">
@@ -5423,23 +4839,23 @@
       <c r="O56">
         <v>19</v>
       </c>
-      <c r="P56" s="4">
+      <c r="P56" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.76893939393939392</v>
       </c>
-      <c r="Q56" s="3">
+      <c r="Q56" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.74</v>
       </c>
-      <c r="R56" s="3">
+      <c r="R56" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.82191780821917804</v>
       </c>
-      <c r="S56" s="3">
+      <c r="S56" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.75824175824175821</v>
       </c>
-      <c r="T56" s="5">
+      <c r="T56">
         <f>+output[[#This Row],[Rechazados acumulados]]-O55</f>
         <v>2</v>
       </c>
@@ -5475,7 +4891,7 @@
       <c r="J57">
         <v>10</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57">
         <v>91</v>
       </c>
       <c r="L57">
@@ -5490,23 +4906,23 @@
       <c r="O57">
         <v>22</v>
       </c>
-      <c r="P57" s="4">
+      <c r="P57" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.99621212121212122</v>
       </c>
-      <c r="Q57" s="3">
+      <c r="Q57" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.99</v>
       </c>
-      <c r="R57" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S57" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T57" s="5">
+      <c r="R57" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S57" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T57">
         <f>+output[[#This Row],[Rechazados acumulados]]-O56</f>
         <v>3</v>
       </c>
@@ -5542,7 +4958,7 @@
       <c r="J58">
         <v>9</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58">
         <v>91</v>
       </c>
       <c r="L58">
@@ -5557,23 +4973,23 @@
       <c r="O58">
         <v>22</v>
       </c>
-      <c r="P58" s="4">
-        <f>+output[[#This Row],[OcupTotal]]/264</f>
-        <v>1</v>
-      </c>
-      <c r="Q58" s="3">
-        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
-        <v>1</v>
-      </c>
-      <c r="R58" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S58" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T58" s="5">
+      <c r="P58" s="2">
+        <f>+output[[#This Row],[OcupTotal]]/264</f>
+        <v>1</v>
+      </c>
+      <c r="Q58" s="2">
+        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
+        <v>1</v>
+      </c>
+      <c r="R58" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S58" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T58">
         <f>+output[[#This Row],[Rechazados acumulados]]-O57</f>
         <v>0</v>
       </c>
@@ -5609,7 +5025,7 @@
       <c r="J59">
         <v>13</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59">
         <v>91</v>
       </c>
       <c r="L59">
@@ -5624,23 +5040,23 @@
       <c r="O59">
         <v>22</v>
       </c>
-      <c r="P59" s="4">
-        <f>+output[[#This Row],[OcupTotal]]/264</f>
-        <v>1</v>
-      </c>
-      <c r="Q59" s="3">
-        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
-        <v>1</v>
-      </c>
-      <c r="R59" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S59" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T59" s="5">
+      <c r="P59" s="2">
+        <f>+output[[#This Row],[OcupTotal]]/264</f>
+        <v>1</v>
+      </c>
+      <c r="Q59" s="2">
+        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
+        <v>1</v>
+      </c>
+      <c r="R59" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S59" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T59">
         <f>+output[[#This Row],[Rechazados acumulados]]-O58</f>
         <v>0</v>
       </c>
@@ -5676,7 +5092,7 @@
       <c r="J60">
         <v>22</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60">
         <v>79</v>
       </c>
       <c r="L60">
@@ -5691,23 +5107,23 @@
       <c r="O60">
         <v>22</v>
       </c>
-      <c r="P60" s="4">
+      <c r="P60" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.95454545454545459</v>
       </c>
-      <c r="Q60" s="3">
-        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
-        <v>1</v>
-      </c>
-      <c r="R60" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S60" s="3">
+      <c r="Q60" s="2">
+        <f>+output[[#This Row],[Ocupación Externo]]/100</f>
+        <v>1</v>
+      </c>
+      <c r="R60" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S60" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.86813186813186816</v>
       </c>
-      <c r="T60" s="5">
+      <c r="T60">
         <f>+output[[#This Row],[Rechazados acumulados]]-O59</f>
         <v>0</v>
       </c>
@@ -5770,11 +5186,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.86301369863013699</v>
       </c>
-      <c r="S61" s="5">
+      <c r="S61">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.60439560439560436</v>
       </c>
-      <c r="T61" s="5">
+      <c r="T61">
         <f>+output[[#This Row],[Rechazados acumulados]]-O60</f>
         <v>0</v>
       </c>
@@ -5837,11 +5253,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.58904109589041098</v>
       </c>
-      <c r="S62" s="5">
+      <c r="S62">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.46153846153846156</v>
       </c>
-      <c r="T62" s="5">
+      <c r="T62">
         <f>+output[[#This Row],[Rechazados acumulados]]-O61</f>
         <v>0</v>
       </c>
@@ -5904,11 +5320,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.41095890410958902</v>
       </c>
-      <c r="S63" s="5">
+      <c r="S63">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.2967032967032967</v>
       </c>
-      <c r="T63" s="5">
+      <c r="T63">
         <f>+output[[#This Row],[Rechazados acumulados]]-O62</f>
         <v>0</v>
       </c>
@@ -5971,11 +5387,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.24657534246575341</v>
       </c>
-      <c r="S64" s="5">
+      <c r="S64">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>8.7912087912087919E-2</v>
       </c>
-      <c r="T64" s="5">
+      <c r="T64">
         <f>+output[[#This Row],[Rechazados acumulados]]-O63</f>
         <v>0</v>
       </c>
@@ -6038,11 +5454,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>6.8493150684931503E-2</v>
       </c>
-      <c r="S65" s="5">
+      <c r="S65">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>3.2967032967032968E-2</v>
       </c>
-      <c r="T65" s="5">
+      <c r="T65">
         <f>+output[[#This Row],[Rechazados acumulados]]-O64</f>
         <v>0</v>
       </c>
@@ -6105,11 +5521,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>2.7397260273972601E-2</v>
       </c>
-      <c r="S66" s="5">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>0</v>
-      </c>
-      <c r="T66" s="5">
+      <c r="S66">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>0</v>
+      </c>
+      <c r="T66">
         <f>+output[[#This Row],[Rechazados acumulados]]-O65</f>
         <v>0</v>
       </c>
@@ -6172,11 +5588,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0</v>
       </c>
-      <c r="S67" s="5">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>0</v>
-      </c>
-      <c r="T67" s="5">
+      <c r="S67">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>0</v>
+      </c>
+      <c r="T67">
         <f>+output[[#This Row],[Rechazados acumulados]]-O66</f>
         <v>0</v>
       </c>
@@ -6212,7 +5628,7 @@
       <c r="J68">
         <v>0</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68">
         <v>24</v>
       </c>
       <c r="L68">
@@ -6227,23 +5643,23 @@
       <c r="O68">
         <v>24</v>
       </c>
-      <c r="P68" s="4">
+      <c r="P68" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.32575757575757575</v>
       </c>
-      <c r="Q68" s="3">
+      <c r="Q68" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.39</v>
       </c>
-      <c r="R68" s="3">
+      <c r="R68" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.31506849315068491</v>
       </c>
-      <c r="S68" s="3">
+      <c r="S68" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.26373626373626374</v>
       </c>
-      <c r="T68" s="5">
+      <c r="T68">
         <f>+output[[#This Row],[Rechazados acumulados]]-O67</f>
         <v>2</v>
       </c>
@@ -6279,7 +5695,7 @@
       <c r="J69">
         <v>0</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69">
         <v>45</v>
       </c>
       <c r="L69">
@@ -6294,23 +5710,23 @@
       <c r="O69">
         <v>25</v>
       </c>
-      <c r="P69" s="4">
+      <c r="P69" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.54166666666666663</v>
       </c>
-      <c r="Q69" s="3">
+      <c r="Q69" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.6</v>
       </c>
-      <c r="R69" s="3">
+      <c r="R69" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.52054794520547942</v>
       </c>
-      <c r="S69" s="3">
+      <c r="S69" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.49450549450549453</v>
       </c>
-      <c r="T69" s="5">
+      <c r="T69">
         <f>+output[[#This Row],[Rechazados acumulados]]-O68</f>
         <v>1</v>
       </c>
@@ -6346,7 +5762,7 @@
       <c r="J70">
         <v>0</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70">
         <v>63</v>
       </c>
       <c r="L70">
@@ -6361,23 +5777,23 @@
       <c r="O70">
         <v>26</v>
       </c>
-      <c r="P70" s="4">
+      <c r="P70" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.69318181818181823</v>
       </c>
-      <c r="Q70" s="3">
+      <c r="Q70" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.76</v>
       </c>
-      <c r="R70" s="3">
+      <c r="R70" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.60273972602739723</v>
       </c>
-      <c r="S70" s="3">
+      <c r="S70" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.69230769230769229</v>
       </c>
-      <c r="T70" s="5">
+      <c r="T70">
         <f>+output[[#This Row],[Rechazados acumulados]]-O69</f>
         <v>1</v>
       </c>
@@ -6413,7 +5829,7 @@
       <c r="J71">
         <v>8</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71">
         <v>72</v>
       </c>
       <c r="L71">
@@ -6428,23 +5844,23 @@
       <c r="O71">
         <v>26</v>
       </c>
-      <c r="P71" s="4">
+      <c r="P71" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.78787878787878785</v>
       </c>
-      <c r="Q71" s="3">
+      <c r="Q71" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.83</v>
       </c>
-      <c r="R71" s="3">
+      <c r="R71" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.72602739726027399</v>
       </c>
-      <c r="S71" s="3">
+      <c r="S71" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.79120879120879117</v>
       </c>
-      <c r="T71" s="5">
+      <c r="T71">
         <f>+output[[#This Row],[Rechazados acumulados]]-O70</f>
         <v>0</v>
       </c>
@@ -6480,7 +5896,7 @@
       <c r="J72">
         <v>8</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72">
         <v>76</v>
       </c>
       <c r="L72">
@@ -6495,23 +5911,23 @@
       <c r="O72">
         <v>28</v>
       </c>
-      <c r="P72" s="4">
+      <c r="P72" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.80681818181818177</v>
       </c>
-      <c r="Q72" s="3">
+      <c r="Q72" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.81</v>
       </c>
-      <c r="R72" s="3">
+      <c r="R72" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.76712328767123283</v>
       </c>
-      <c r="S72" s="3">
+      <c r="S72" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.8351648351648352</v>
       </c>
-      <c r="T72" s="5">
+      <c r="T72">
         <f>+output[[#This Row],[Rechazados acumulados]]-O71</f>
         <v>2</v>
       </c>
@@ -6547,7 +5963,7 @@
       <c r="J73">
         <v>18</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73">
         <v>63</v>
       </c>
       <c r="L73">
@@ -6562,23 +5978,23 @@
       <c r="O73">
         <v>28</v>
       </c>
-      <c r="P73" s="4">
+      <c r="P73" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.70833333333333337</v>
       </c>
-      <c r="Q73" s="3">
+      <c r="Q73" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.7</v>
       </c>
-      <c r="R73" s="3">
+      <c r="R73" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.73972602739726023</v>
       </c>
-      <c r="S73" s="3">
+      <c r="S73" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.69230769230769229</v>
       </c>
-      <c r="T73" s="5">
+      <c r="T73">
         <f>+output[[#This Row],[Rechazados acumulados]]-O72</f>
         <v>0</v>
       </c>
@@ -6614,7 +6030,7 @@
       <c r="J74">
         <v>15</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74">
         <v>59</v>
       </c>
       <c r="L74">
@@ -6629,23 +6045,23 @@
       <c r="O74">
         <v>28</v>
       </c>
-      <c r="P74" s="4">
+      <c r="P74" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.625</v>
       </c>
-      <c r="Q74" s="3">
+      <c r="Q74" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.64</v>
       </c>
-      <c r="R74" s="3">
+      <c r="R74" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.57534246575342463</v>
       </c>
-      <c r="S74" s="3">
+      <c r="S74" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.64835164835164838</v>
       </c>
-      <c r="T74" s="5">
+      <c r="T74">
         <f>+output[[#This Row],[Rechazados acumulados]]-O73</f>
         <v>0</v>
       </c>
@@ -6681,7 +6097,7 @@
       <c r="J75">
         <v>17</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75">
         <v>56</v>
       </c>
       <c r="L75">
@@ -6696,23 +6112,23 @@
       <c r="O75">
         <v>28</v>
       </c>
-      <c r="P75" s="4">
+      <c r="P75" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.61363636363636365</v>
       </c>
-      <c r="Q75" s="3">
+      <c r="Q75" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.59</v>
       </c>
-      <c r="R75" s="3">
+      <c r="R75" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.64383561643835618</v>
       </c>
-      <c r="S75" s="3">
+      <c r="S75" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.61538461538461542</v>
       </c>
-      <c r="T75" s="5">
+      <c r="T75">
         <f>+output[[#This Row],[Rechazados acumulados]]-O74</f>
         <v>0</v>
       </c>
@@ -6748,7 +6164,7 @@
       <c r="J76">
         <v>11</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76">
         <v>61</v>
       </c>
       <c r="L76">
@@ -6763,23 +6179,23 @@
       <c r="O76">
         <v>28</v>
       </c>
-      <c r="P76" s="4">
+      <c r="P76" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.59469696969696972</v>
       </c>
-      <c r="Q76" s="3">
+      <c r="Q76" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.54</v>
       </c>
-      <c r="R76" s="3">
+      <c r="R76" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.57534246575342463</v>
       </c>
-      <c r="S76" s="3">
+      <c r="S76" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.67032967032967028</v>
       </c>
-      <c r="T76" s="5">
+      <c r="T76">
         <f>+output[[#This Row],[Rechazados acumulados]]-O75</f>
         <v>0</v>
       </c>
@@ -6815,7 +6231,7 @@
       <c r="J77">
         <v>14</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77">
         <v>70</v>
       </c>
       <c r="L77">
@@ -6830,23 +6246,23 @@
       <c r="O77">
         <v>31</v>
       </c>
-      <c r="P77" s="4">
+      <c r="P77" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.68181818181818177</v>
       </c>
-      <c r="Q77" s="3">
+      <c r="Q77" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="R77" s="3">
+      <c r="R77" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.75342465753424659</v>
       </c>
-      <c r="S77" s="3">
+      <c r="S77" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.76923076923076927</v>
       </c>
-      <c r="T77" s="5">
+      <c r="T77">
         <f>+output[[#This Row],[Rechazados acumulados]]-O76</f>
         <v>3</v>
       </c>
@@ -6882,7 +6298,7 @@
       <c r="J78">
         <v>10</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78">
         <v>85</v>
       </c>
       <c r="L78">
@@ -6897,23 +6313,23 @@
       <c r="O78">
         <v>32</v>
       </c>
-      <c r="P78" s="4">
+      <c r="P78" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.84848484848484851</v>
       </c>
-      <c r="Q78" s="3">
+      <c r="Q78" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.74</v>
       </c>
-      <c r="R78" s="3">
+      <c r="R78" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.8904109589041096</v>
       </c>
-      <c r="S78" s="3">
+      <c r="S78" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.93406593406593408</v>
       </c>
-      <c r="T78" s="5">
+      <c r="T78">
         <f>+output[[#This Row],[Rechazados acumulados]]-O77</f>
         <v>1</v>
       </c>
@@ -6949,7 +6365,7 @@
       <c r="J79">
         <v>8</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79">
         <v>91</v>
       </c>
       <c r="L79">
@@ -6964,23 +6380,23 @@
       <c r="O79">
         <v>33</v>
       </c>
-      <c r="P79" s="4">
+      <c r="P79" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.9507575757575758</v>
       </c>
-      <c r="Q79" s="3">
+      <c r="Q79" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.87</v>
       </c>
-      <c r="R79" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S79" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T79" s="5">
+      <c r="R79" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S79" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T79">
         <f>+output[[#This Row],[Rechazados acumulados]]-O78</f>
         <v>1</v>
       </c>
@@ -7016,7 +6432,7 @@
       <c r="J80">
         <v>18</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80">
         <v>91</v>
       </c>
       <c r="L80">
@@ -7031,23 +6447,23 @@
       <c r="O80">
         <v>34</v>
       </c>
-      <c r="P80" s="4">
+      <c r="P80" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.97348484848484851</v>
       </c>
-      <c r="Q80" s="3">
+      <c r="Q80" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.93</v>
       </c>
-      <c r="R80" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S80" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T80" s="5">
+      <c r="R80" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S80" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T80">
         <f>+output[[#This Row],[Rechazados acumulados]]-O79</f>
         <v>1</v>
       </c>
@@ -7083,7 +6499,7 @@
       <c r="J81">
         <v>13</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81">
         <v>91</v>
       </c>
       <c r="L81">
@@ -7098,23 +6514,23 @@
       <c r="O81">
         <v>34</v>
       </c>
-      <c r="P81" s="4">
+      <c r="P81" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.96590909090909094</v>
       </c>
-      <c r="Q81" s="3">
+      <c r="Q81" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.91</v>
       </c>
-      <c r="R81" s="3">
-        <f>+output[[#This Row],[Ocupación Central]]/73</f>
-        <v>1</v>
-      </c>
-      <c r="S81" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T81" s="5">
+      <c r="R81" s="2">
+        <f>+output[[#This Row],[Ocupación Central]]/73</f>
+        <v>1</v>
+      </c>
+      <c r="S81" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T81">
         <f>+output[[#This Row],[Rechazados acumulados]]-O80</f>
         <v>0</v>
       </c>
@@ -7150,7 +6566,7 @@
       <c r="J82">
         <v>23</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82">
         <v>74</v>
       </c>
       <c r="L82">
@@ -7165,23 +6581,23 @@
       <c r="O82">
         <v>34</v>
       </c>
-      <c r="P82" s="4">
+      <c r="P82" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.73863636363636365</v>
       </c>
-      <c r="Q82" s="3">
+      <c r="Q82" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.73</v>
       </c>
-      <c r="R82" s="3">
+      <c r="R82" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.65753424657534243</v>
       </c>
-      <c r="S82" s="3">
+      <c r="S82" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.81318681318681318</v>
       </c>
-      <c r="T82" s="5">
+      <c r="T82">
         <f>+output[[#This Row],[Rechazados acumulados]]-O81</f>
         <v>0</v>
       </c>
@@ -7244,11 +6660,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.49315068493150682</v>
       </c>
-      <c r="S83" s="5">
+      <c r="S83">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.59340659340659341</v>
       </c>
-      <c r="T83" s="5">
+      <c r="T83">
         <f>+output[[#This Row],[Rechazados acumulados]]-O82</f>
         <v>0</v>
       </c>
@@ -7311,11 +6727,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.38356164383561642</v>
       </c>
-      <c r="S84" s="5">
+      <c r="S84">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.37362637362637363</v>
       </c>
-      <c r="T84" s="5">
+      <c r="T84">
         <f>+output[[#This Row],[Rechazados acumulados]]-O83</f>
         <v>0</v>
       </c>
@@ -7378,11 +6794,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.20547945205479451</v>
       </c>
-      <c r="S85" s="5">
+      <c r="S85">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.18681318681318682</v>
       </c>
-      <c r="T85" s="5">
+      <c r="T85">
         <f>+output[[#This Row],[Rechazados acumulados]]-O84</f>
         <v>0</v>
       </c>
@@ -7445,11 +6861,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>2.7397260273972601E-2</v>
       </c>
-      <c r="S86" s="5">
+      <c r="S86">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>9.8901098901098897E-2</v>
       </c>
-      <c r="T86" s="5">
+      <c r="T86">
         <f>+output[[#This Row],[Rechazados acumulados]]-O85</f>
         <v>0</v>
       </c>
@@ -7512,11 +6928,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>1.3698630136986301E-2</v>
       </c>
-      <c r="S87" s="5">
+      <c r="S87">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>3.2967032967032968E-2</v>
       </c>
-      <c r="T87" s="5">
+      <c r="T87">
         <f>+output[[#This Row],[Rechazados acumulados]]-O86</f>
         <v>0</v>
       </c>
@@ -7579,11 +6995,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0</v>
       </c>
-      <c r="S88" s="5">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>0</v>
-      </c>
-      <c r="T88" s="5">
+      <c r="S88">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>0</v>
+      </c>
+      <c r="T88">
         <f>+output[[#This Row],[Rechazados acumulados]]-O87</f>
         <v>0</v>
       </c>
@@ -7646,11 +7062,11 @@
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0</v>
       </c>
-      <c r="S89" s="5">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>0</v>
-      </c>
-      <c r="T89" s="5">
+      <c r="S89">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>0</v>
+      </c>
+      <c r="T89">
         <f>+output[[#This Row],[Rechazados acumulados]]-O88</f>
         <v>0</v>
       </c>
@@ -7686,7 +7102,7 @@
       <c r="J90">
         <v>0</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90">
         <v>35</v>
       </c>
       <c r="L90">
@@ -7701,23 +7117,23 @@
       <c r="O90">
         <v>36</v>
       </c>
-      <c r="P90" s="4">
+      <c r="P90" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.32196969696969696</v>
       </c>
-      <c r="Q90" s="3">
+      <c r="Q90" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.28000000000000003</v>
       </c>
-      <c r="R90" s="3">
+      <c r="R90" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.30136986301369861</v>
       </c>
-      <c r="S90" s="3">
+      <c r="S90" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.38461538461538464</v>
       </c>
-      <c r="T90" s="5">
+      <c r="T90">
         <f>+output[[#This Row],[Rechazados acumulados]]-O89</f>
         <v>2</v>
       </c>
@@ -7753,7 +7169,7 @@
       <c r="J91">
         <v>0</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91">
         <v>61</v>
       </c>
       <c r="L91">
@@ -7768,23 +7184,23 @@
       <c r="O91">
         <v>36</v>
       </c>
-      <c r="P91" s="4">
+      <c r="P91" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.54545454545454541</v>
       </c>
-      <c r="Q91" s="3">
+      <c r="Q91" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.49</v>
       </c>
-      <c r="R91" s="3">
+      <c r="R91" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.46575342465753422</v>
       </c>
-      <c r="S91" s="3">
+      <c r="S91" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.67032967032967028</v>
       </c>
-      <c r="T91" s="5">
+      <c r="T91">
         <f>+output[[#This Row],[Rechazados acumulados]]-O90</f>
         <v>0</v>
       </c>
@@ -7820,7 +7236,7 @@
       <c r="J92">
         <v>1</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92">
         <v>71</v>
       </c>
       <c r="L92">
@@ -7835,23 +7251,23 @@
       <c r="O92">
         <v>36</v>
       </c>
-      <c r="P92" s="4">
+      <c r="P92" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.64772727272727271</v>
       </c>
-      <c r="Q92" s="3">
+      <c r="Q92" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.6</v>
       </c>
-      <c r="R92" s="3">
+      <c r="R92" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.54794520547945202</v>
       </c>
-      <c r="S92" s="3">
+      <c r="S92" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.78021978021978022</v>
       </c>
-      <c r="T92" s="5">
+      <c r="T92">
         <f>+output[[#This Row],[Rechazados acumulados]]-O91</f>
         <v>0</v>
       </c>
@@ -7887,7 +7303,7 @@
       <c r="J93">
         <v>1</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93">
         <v>81</v>
       </c>
       <c r="L93">
@@ -7902,23 +7318,23 @@
       <c r="O93">
         <v>37</v>
       </c>
-      <c r="P93" s="4">
+      <c r="P93" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.76893939393939392</v>
       </c>
-      <c r="Q93" s="3">
+      <c r="Q93" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.7</v>
       </c>
-      <c r="R93" s="3">
+      <c r="R93" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.71232876712328763</v>
       </c>
-      <c r="S93" s="3">
+      <c r="S93" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.89010989010989006</v>
       </c>
-      <c r="T93" s="5">
+      <c r="T93">
         <f>+output[[#This Row],[Rechazados acumulados]]-O92</f>
         <v>1</v>
       </c>
@@ -7954,7 +7370,7 @@
       <c r="J94">
         <v>12</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94">
         <v>82</v>
       </c>
       <c r="L94">
@@ -7969,23 +7385,23 @@
       <c r="O94">
         <v>37</v>
       </c>
-      <c r="P94" s="4">
+      <c r="P94" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.78409090909090906</v>
       </c>
-      <c r="Q94" s="3">
+      <c r="Q94" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.72</v>
       </c>
-      <c r="R94" s="3">
+      <c r="R94" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.72602739726027399</v>
       </c>
-      <c r="S94" s="3">
+      <c r="S94" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.90109890109890112</v>
       </c>
-      <c r="T94" s="5">
+      <c r="T94">
         <f>+output[[#This Row],[Rechazados acumulados]]-O93</f>
         <v>0</v>
       </c>
@@ -8021,7 +7437,7 @@
       <c r="J95">
         <v>20</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95">
         <v>75</v>
       </c>
       <c r="L95">
@@ -8036,23 +7452,23 @@
       <c r="O95">
         <v>37</v>
       </c>
-      <c r="P95" s="4">
+      <c r="P95" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.66287878787878785</v>
       </c>
-      <c r="Q95" s="3">
+      <c r="Q95" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.56000000000000005</v>
       </c>
-      <c r="R95" s="3">
+      <c r="R95" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.60273972602739723</v>
       </c>
-      <c r="S95" s="3">
+      <c r="S95" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.82417582417582413</v>
       </c>
-      <c r="T95" s="5">
+      <c r="T95">
         <f>+output[[#This Row],[Rechazados acumulados]]-O94</f>
         <v>0</v>
       </c>
@@ -8088,7 +7504,7 @@
       <c r="J96">
         <v>19</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96">
         <v>62</v>
       </c>
       <c r="L96">
@@ -8103,23 +7519,23 @@
       <c r="O96">
         <v>37</v>
       </c>
-      <c r="P96" s="4">
+      <c r="P96" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.57196969696969702</v>
       </c>
-      <c r="Q96" s="3">
+      <c r="Q96" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.49</v>
       </c>
-      <c r="R96" s="3">
+      <c r="R96" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.54794520547945202</v>
       </c>
-      <c r="S96" s="3">
+      <c r="S96" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.68131868131868134</v>
       </c>
-      <c r="T96" s="5">
+      <c r="T96">
         <f>+output[[#This Row],[Rechazados acumulados]]-O95</f>
         <v>0</v>
       </c>
@@ -8155,7 +7571,7 @@
       <c r="J97">
         <v>16</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97">
         <v>65</v>
       </c>
       <c r="L97">
@@ -8170,23 +7586,23 @@
       <c r="O97">
         <v>37</v>
       </c>
-      <c r="P97" s="4">
+      <c r="P97" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.54166666666666663</v>
       </c>
-      <c r="Q97" s="3">
+      <c r="Q97" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.41</v>
       </c>
-      <c r="R97" s="3">
+      <c r="R97" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.50684931506849318</v>
       </c>
-      <c r="S97" s="3">
+      <c r="S97" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.7142857142857143</v>
       </c>
-      <c r="T97" s="5">
+      <c r="T97">
         <f>+output[[#This Row],[Rechazados acumulados]]-O96</f>
         <v>0</v>
       </c>
@@ -8222,7 +7638,7 @@
       <c r="J98">
         <v>13</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98">
         <v>65</v>
       </c>
       <c r="L98">
@@ -8237,23 +7653,23 @@
       <c r="O98">
         <v>37</v>
       </c>
-      <c r="P98" s="4">
+      <c r="P98" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.49242424242424243</v>
       </c>
-      <c r="Q98" s="3">
+      <c r="Q98" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.36</v>
       </c>
-      <c r="R98" s="3">
+      <c r="R98" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.39726027397260272</v>
       </c>
-      <c r="S98" s="3">
+      <c r="S98" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.7142857142857143</v>
       </c>
-      <c r="T98" s="5">
+      <c r="T98">
         <f>+output[[#This Row],[Rechazados acumulados]]-O97</f>
         <v>0</v>
       </c>
@@ -8289,7 +7705,7 @@
       <c r="J99">
         <v>14</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99">
         <v>72</v>
       </c>
       <c r="L99">
@@ -8304,23 +7720,23 @@
       <c r="O99">
         <v>37</v>
       </c>
-      <c r="P99" s="4">
+      <c r="P99" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.53787878787878785</v>
       </c>
-      <c r="Q99" s="3">
+      <c r="Q99" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.37</v>
       </c>
-      <c r="R99" s="3">
+      <c r="R99" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.45205479452054792</v>
       </c>
-      <c r="S99" s="3">
+      <c r="S99" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.79120879120879117</v>
       </c>
-      <c r="T99" s="5">
+      <c r="T99">
         <f>+output[[#This Row],[Rechazados acumulados]]-O98</f>
         <v>0</v>
       </c>
@@ -8356,7 +7772,7 @@
       <c r="J100">
         <v>17</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100">
         <v>86</v>
       </c>
       <c r="L100">
@@ -8371,23 +7787,23 @@
       <c r="O100">
         <v>44</v>
       </c>
-      <c r="P100" s="4">
+      <c r="P100" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.76893939393939392</v>
       </c>
-      <c r="Q100" s="3">
+      <c r="Q100" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.66</v>
       </c>
-      <c r="R100" s="3">
+      <c r="R100" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.69863013698630139</v>
       </c>
-      <c r="S100" s="3">
+      <c r="S100" s="2">
         <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
         <v>0.94505494505494503</v>
       </c>
-      <c r="T100" s="5">
+      <c r="T100">
         <f>+output[[#This Row],[Rechazados acumulados]]-O99</f>
         <v>7</v>
       </c>
@@ -8423,7 +7839,7 @@
       <c r="J101">
         <v>12</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101">
         <v>91</v>
       </c>
       <c r="L101">
@@ -8438,23 +7854,23 @@
       <c r="O101">
         <v>47</v>
       </c>
-      <c r="P101" s="4">
+      <c r="P101" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.91287878787878785</v>
       </c>
-      <c r="Q101" s="3">
+      <c r="Q101" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.89</v>
       </c>
-      <c r="R101" s="3">
+      <c r="R101" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.83561643835616439</v>
       </c>
-      <c r="S101" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T101" s="5">
+      <c r="S101" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T101">
         <f>+output[[#This Row],[Rechazados acumulados]]-O100</f>
         <v>3</v>
       </c>
@@ -8490,7 +7906,7 @@
       <c r="J102">
         <v>17</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102">
         <v>91</v>
       </c>
       <c r="L102">
@@ -8505,23 +7921,23 @@
       <c r="O102">
         <v>47</v>
       </c>
-      <c r="P102" s="4">
+      <c r="P102" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.93181818181818177</v>
       </c>
-      <c r="Q102" s="3">
+      <c r="Q102" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.93</v>
       </c>
-      <c r="R102" s="3">
+      <c r="R102" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.84931506849315064</v>
       </c>
-      <c r="S102" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T102" s="5">
+      <c r="S102" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T102">
         <f>+output[[#This Row],[Rechazados acumulados]]-O101</f>
         <v>0</v>
       </c>
@@ -8557,7 +7973,7 @@
       <c r="J103">
         <v>12</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103">
         <v>91</v>
       </c>
       <c r="L103">
@@ -8572,23 +7988,23 @@
       <c r="O103">
         <v>47</v>
       </c>
-      <c r="P103" s="4">
+      <c r="P103" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.93560606060606055</v>
       </c>
-      <c r="Q103" s="3">
+      <c r="Q103" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.96</v>
       </c>
-      <c r="R103" s="3">
+      <c r="R103" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.82191780821917804</v>
       </c>
-      <c r="S103" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T103" s="5">
+      <c r="S103" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T103">
         <f>+output[[#This Row],[Rechazados acumulados]]-O102</f>
         <v>0</v>
       </c>
@@ -8624,7 +8040,7 @@
       <c r="J104">
         <v>7</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104">
         <v>91</v>
       </c>
       <c r="L104">
@@ -8639,99 +8055,77 @@
       <c r="O104">
         <v>47</v>
       </c>
-      <c r="P104" s="4">
+      <c r="P104" s="2">
         <f>+output[[#This Row],[OcupTotal]]/264</f>
         <v>0.90530303030303028</v>
       </c>
-      <c r="Q104" s="3">
+      <c r="Q104" s="2">
         <f>+output[[#This Row],[Ocupación Externo]]/100</f>
         <v>0.9</v>
       </c>
-      <c r="R104" s="3">
+      <c r="R104" s="2">
         <f>+output[[#This Row],[Ocupación Central]]/73</f>
         <v>0.79452054794520544</v>
       </c>
-      <c r="S104" s="3">
-        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
-        <v>1</v>
-      </c>
-      <c r="T104" s="5">
+      <c r="S104" s="2">
+        <f>+output[[#This Row],[Ocupación Polideportivo]]/91</f>
+        <v>1</v>
+      </c>
+      <c r="T104">
         <f>+output[[#This Row],[Rechazados acumulados]]-O103</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="N2:N104">
-    <cfRule type="cellIs" dxfId="26" priority="14" operator="equal">
-      <formula>264</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="cellIs" dxfId="25" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="15" operator="equal">
       <formula>100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:H1048576">
-    <cfRule type="cellIs" dxfId="24" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="14" operator="equal">
       <formula>73</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="cellIs" dxfId="23" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="13" operator="equal">
       <formula>91</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P1:P1048576">
-    <cfRule type="cellIs" dxfId="22" priority="10" operator="between">
+  <conditionalFormatting sqref="N2:N104">
+    <cfRule type="cellIs" dxfId="15" priority="16" operator="equal">
+      <formula>264</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P1:Q1048576">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="between">
       <formula>0.5</formula>
       <formula>0.75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P1048576">
-    <cfRule type="cellIs" dxfId="21" priority="9" operator="greaterThan">
+  <conditionalFormatting sqref="P2:R1048576">
+    <cfRule type="cellIs" dxfId="13" priority="7" operator="greaterThan">
       <formula>0.75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q1:Q1048576">
-    <cfRule type="cellIs" dxfId="20" priority="8" operator="between">
+  <conditionalFormatting sqref="R2:R1048576">
+    <cfRule type="cellIs" dxfId="12" priority="8" operator="between">
       <formula>0.5</formula>
       <formula>0.75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q1048576">
-    <cfRule type="cellIs" dxfId="19" priority="7" operator="greaterThan">
-      <formula>0.75</formula>
+  <conditionalFormatting sqref="T2:T104">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="greaterThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R1048576">
-    <cfRule type="cellIs" dxfId="18" priority="6" operator="between">
+  <conditionalFormatting sqref="S2:S1048576">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="between">
       <formula>0.5</formula>
       <formula>0.75</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0.75</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S1048576">
-    <cfRule type="cellIs" dxfId="16" priority="4" operator="between">
-      <formula>0.5</formula>
-      <formula>0.75</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S104">
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="between">
-      <formula>0.5</formula>
-      <formula>75</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S104">
-    <cfRule type="cellIs" dxfId="14" priority="2" operator="greaterThan">
-      <formula>0.75</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T104">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>